<commit_message>
Add site property field, discard-record flow, and document completed Fulcrum migration
Site records now capture pastoral station (property) alongside NTA, matching
the entity properties added to Central during the Fulcrum migration; the
record sheet gains a discard button (continue timing vs. reset-and-discard)
for aborted searches. Docs updated to reflect the migration having actually
run against live Central: FULCRUM_MIGRATION.md now has the confirmed
procedure and property mapping table, and CLAUDE.md's entities section
records what that run verified (baseVersion/trunkVersion/branchId acceptance)
versus what's still unexercised through the app's own app-user OpenRosa path
(manifest CSV attachment, create="true" entity registration).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/toad_detection_survey.xlsx
+++ b/toad_detection_survey.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,39 +737,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one property_choices</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>visit_date</t>
+          <t>property</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>${is_new_site} = 'yes'</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>property</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>visit_time</t>
+          <t>visit_date</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -781,17 +791,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>time</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>temperature_c</t>
+          <t>visit_time</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Temperature (°C)</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -803,17 +813,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>select_one yn_choices</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>toads_access_water</t>
+          <t>temperature_c</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Can toads access the water?</t>
+          <t>Temperature (°C)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -825,17 +835,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one yn_choices</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>people_searching</t>
+          <t>toads_access_water</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>How many people searching?</t>
+          <t>Can toads access the water?</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -852,17 +862,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>time_searched_minutes</t>
+          <t>people_searching</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Time searched (minutes)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Time taken to detect a toad, or total search time if none found</t>
+          <t>How many people searching?</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -874,17 +879,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>select_one yn_choices</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>toad_found</t>
+          <t>time_searched_minutes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Was a toad found?</t>
+          <t>Time searched (minutes)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Time taken to detect a toad, or total search time if none found</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -896,20 +906,42 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>select_one yn_choices</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>toad_found</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Was a toad found?</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -926,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1249,6 +1281,227 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>Nyamal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Not on a known property</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PROP-FDS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Frazier Downs Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PROP-SHAMS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Shamrock Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PROP-APS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Anna Plains Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PROP-NDS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Nita Downs Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PROP-SHAMG</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Shamrock Gardens</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PROP-SHEL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Shelamar Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PROP-RPS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Roebuck Plains Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PROP-DD</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dampier Downs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PROP-LIV</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Liveringa</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PROP-MYR</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Myroodah</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PROP-YM</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Yakka Munga</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>property_choices</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PROP-YEE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Yeeda</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switched to timer first, but with optional shortcut to creating a new site (for daytime setup)
</commit_message>
<xml_diff>
--- a/toad_detection_survey.xlsx
+++ b/toad_detection_survey.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -769,17 +769,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one yn_choices</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>visit_date</t>
+          <t>survey_conducted</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Was a timed search actually carried out on this visit?</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -791,17 +791,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>visit_time</t>
+          <t>visit_date</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -813,17 +813,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>time</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>temperature_c</t>
+          <t>visit_time</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Temperature (°C)</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -835,44 +835,54 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>select_one yn_choices</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>toads_access_water</t>
+          <t>temperature_c</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Can toads access the water?</t>
+          <t>Temperature (°C)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one yn_choices</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>people_searching</t>
+          <t>toads_access_water</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>How many people searching?</t>
+          <t>Can toads access the water?</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
         </is>
       </c>
     </row>
@@ -884,64 +894,101 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>time_searched_minutes</t>
+          <t>people_searching</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Time searched (minutes)</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Time taken to detect a toad, or total search time if none found</t>
+          <t>How many people searching?</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>select_one yn_choices</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>toad_found</t>
+          <t>time_searched_minutes</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Was a toad found?</t>
+          <t>Time searched (minutes)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Time taken to detect a toad, or total search time if none found</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>select_one yn_choices</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>toad_found</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Was a toad found?</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>${survey_conducted} = 'yes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>